<commit_message>
final push to make the algos work
</commit_message>
<xml_diff>
--- a/subsystems database.xlsx
+++ b/subsystems database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cdepaor2\Desktop\EUCASS_2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{421765E8-A994-4544-8FA4-8B23D6129513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1497E37-3703-4A5F-A136-DE36226DD7BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-795" windowWidth="29040" windowHeight="15720" xr2:uid="{DA27C19A-18DB-4E19-9AD3-8F88A97C8EE8}"/>
+    <workbookView xWindow="900" yWindow="912" windowWidth="21600" windowHeight="11232" xr2:uid="{DA27C19A-18DB-4E19-9AD3-8F88A97C8EE8}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="29">
   <si>
     <t>md</t>
   </si>
@@ -105,6 +105,24 @@
   </si>
   <si>
     <t>9205-FLO-1-CLS</t>
+  </si>
+  <si>
+    <t>0609-LLPS-GRC</t>
+  </si>
+  <si>
+    <t>ND</t>
+  </si>
+  <si>
+    <t>0610-LAT-1</t>
+  </si>
+  <si>
+    <t>kW</t>
+  </si>
+  <si>
+    <t>kWh</t>
+  </si>
+  <si>
+    <t>mt</t>
   </si>
 </sst>
 </file>
@@ -186,23 +204,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -538,453 +555,646 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66EAA883-65ED-4288-9D11-90A18C3BBAF4}">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="7.28515625" customWidth="1"/>
+    <col min="4" max="11" width="11.5703125" customWidth="1"/>
+    <col min="12" max="12" width="17.85546875" customWidth="1"/>
+    <col min="13" max="13" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="N1" s="5" t="s">
         <v>11</v>
       </c>
+      <c r="O1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B2" s="1">
+        <f>SUM(C2:E2)</f>
+        <v>16448</v>
+      </c>
+      <c r="C2" s="1">
         <v>2373</v>
       </c>
-      <c r="C2" s="1">
+      <c r="D2" s="1">
         <v>5295</v>
       </c>
-      <c r="D2" s="1">
+      <c r="E2" s="1">
         <v>8780</v>
       </c>
-      <c r="E2" s="1">
+      <c r="F2" s="1">
         <v>2265</v>
       </c>
-      <c r="F2" s="1">
+      <c r="G2" s="1">
         <v>311</v>
       </c>
-      <c r="G2" s="2">
+      <c r="H2" s="4">
         <v>460</v>
       </c>
-      <c r="H2" s="1">
+      <c r="I2" s="1">
         <v>495</v>
       </c>
-      <c r="I2" s="1">
+      <c r="J2" s="1">
         <v>366</v>
       </c>
-      <c r="J2" s="1">
+      <c r="K2" s="1">
         <v>29</v>
       </c>
-      <c r="K2" s="1">
+      <c r="L2" s="1">
         <v>404</v>
       </c>
-      <c r="L2" s="1">
+      <c r="M2" s="1">
         <v>273</v>
       </c>
-      <c r="M2" s="1"/>
+      <c r="N2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O2" s="1">
+        <v>0.112</v>
+      </c>
+      <c r="P2">
+        <f>O2*75</f>
+        <v>8.4</v>
+      </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B3" s="1">
+        <f t="shared" ref="B3:B13" si="0">SUM(C3:E3)</f>
+        <v>5038.6000000000004</v>
+      </c>
+      <c r="C3" s="1">
         <v>1673.7</v>
       </c>
-      <c r="C3" s="1">
+      <c r="D3" s="1">
         <v>473.3</v>
       </c>
-      <c r="D3" s="1">
+      <c r="E3" s="1">
         <v>2891.6000000000004</v>
       </c>
-      <c r="E3" s="1">
+      <c r="F3" s="1">
         <v>1822</v>
       </c>
-      <c r="F3" s="1">
+      <c r="G3" s="1">
         <v>333</v>
       </c>
-      <c r="G3" s="2">
+      <c r="H3" s="4">
         <v>532.9</v>
       </c>
-      <c r="H3" s="1">
+      <c r="I3" s="1">
         <v>252.5</v>
       </c>
-      <c r="I3" s="1">
+      <c r="J3" s="1">
         <v>125.7</v>
       </c>
-      <c r="J3" s="1">
+      <c r="K3" s="1">
         <v>120.1</v>
       </c>
-      <c r="K3" s="1">
+      <c r="L3" s="1">
         <v>113.5</v>
       </c>
-      <c r="L3" s="1">
+      <c r="M3" s="1">
         <v>56</v>
       </c>
-      <c r="M3" s="1"/>
+      <c r="N3" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B4" s="1">
+        <f t="shared" si="0"/>
+        <v>60075</v>
+      </c>
+      <c r="C4" s="1">
         <v>9823</v>
       </c>
-      <c r="C4" s="1">
+      <c r="D4" s="1">
         <v>25000</v>
       </c>
-      <c r="D4" s="1">
+      <c r="E4" s="1">
         <v>25252</v>
       </c>
-      <c r="E4" s="1">
+      <c r="F4" s="1">
         <v>2100</v>
       </c>
-      <c r="F4" s="1">
+      <c r="G4" s="1">
         <v>450</v>
       </c>
-      <c r="G4" s="2">
+      <c r="H4" s="4">
         <v>1681</v>
       </c>
-      <c r="H4" s="1">
+      <c r="I4" s="1">
         <v>4258</v>
       </c>
-      <c r="I4" s="1">
+      <c r="J4" s="1">
         <v>478</v>
       </c>
-      <c r="J4" s="1">
+      <c r="K4" s="1">
         <v>934</v>
       </c>
-      <c r="K4" s="1">
+      <c r="L4" s="1">
         <v>2017</v>
       </c>
-      <c r="L4" s="1">
+      <c r="M4" s="1">
         <v>455</v>
       </c>
-      <c r="M4" s="1"/>
+      <c r="N4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O4" s="1">
+        <v>2</v>
+      </c>
+      <c r="P4">
+        <f>O4*3*24</f>
+        <v>144</v>
+      </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="1">
+        <f t="shared" si="0"/>
+        <v>69298</v>
+      </c>
+      <c r="C5" s="1">
         <v>7899</v>
       </c>
-      <c r="C5" s="1">
+      <c r="D5" s="1">
         <v>25000</v>
       </c>
-      <c r="D5" s="1">
+      <c r="E5" s="1">
         <v>36399</v>
       </c>
-      <c r="E5" s="1">
+      <c r="F5" s="1">
         <v>2100</v>
       </c>
-      <c r="F5" s="1">
+      <c r="G5" s="1">
         <v>333</v>
       </c>
-      <c r="G5" s="2">
+      <c r="H5" s="4">
         <v>1955</v>
       </c>
-      <c r="H5" s="1">
+      <c r="I5" s="1">
         <v>2943</v>
       </c>
-      <c r="I5" s="1">
+      <c r="J5" s="1">
         <v>478</v>
       </c>
-      <c r="J5" s="1">
+      <c r="K5" s="1">
         <v>1062</v>
       </c>
-      <c r="K5" s="1">
+      <c r="L5" s="1">
         <v>1006</v>
       </c>
-      <c r="L5" s="1">
+      <c r="M5" s="1">
         <v>455</v>
       </c>
-      <c r="M5" s="1"/>
+      <c r="N5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O5" s="1">
+        <v>2</v>
+      </c>
+      <c r="P5">
+        <f>O5*3*24</f>
+        <v>144</v>
+      </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B6" s="1">
+        <f>SUM(C6:E6)</f>
+        <v>89365</v>
+      </c>
+      <c r="C6" s="1">
         <v>9320</v>
       </c>
-      <c r="C6" s="1">
+      <c r="D6" s="1">
         <v>35894</v>
       </c>
-      <c r="D6" s="1">
+      <c r="E6" s="1">
         <v>44151</v>
       </c>
-      <c r="E6" s="1">
+      <c r="F6" s="1">
         <v>3100</v>
       </c>
-      <c r="F6" s="1">
+      <c r="G6" s="1">
         <v>450</v>
       </c>
-      <c r="G6" s="2">
+      <c r="H6" s="4">
         <v>1770</v>
       </c>
-      <c r="H6" s="1">
+      <c r="I6" s="1">
         <v>4969</v>
       </c>
-      <c r="I6" s="1">
+      <c r="J6" s="1">
         <v>385</v>
       </c>
-      <c r="J6" s="1">
+      <c r="K6" s="1">
         <v>307</v>
       </c>
-      <c r="K6" s="1">
+      <c r="L6" s="1">
         <v>420</v>
       </c>
-      <c r="L6" s="1">
+      <c r="M6" s="1">
         <v>1469</v>
       </c>
-      <c r="M6" s="1">
+      <c r="N6" s="1">
         <v>1878</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B7" s="1">
+        <f t="shared" si="0"/>
+        <v>44821</v>
+      </c>
+      <c r="C7" s="1">
         <v>5858</v>
       </c>
-      <c r="C7" s="1">
+      <c r="D7" s="1">
         <v>16461</v>
       </c>
-      <c r="D7" s="1">
+      <c r="E7" s="1">
         <v>22502</v>
       </c>
-      <c r="E7" s="1">
+      <c r="F7" s="1">
         <v>2260</v>
       </c>
-      <c r="F7" s="1">
+      <c r="G7" s="1">
         <v>379</v>
       </c>
-      <c r="G7" s="2">
+      <c r="H7" s="4">
         <v>2822</v>
       </c>
-      <c r="H7" s="1">
+      <c r="I7" s="1">
         <v>1749</v>
       </c>
-      <c r="I7" s="1">
+      <c r="J7" s="1">
         <v>204</v>
       </c>
-      <c r="J7" s="1">
+      <c r="K7" s="1">
         <v>818</v>
       </c>
-      <c r="K7" s="1">
+      <c r="L7" s="1">
         <v>265</v>
       </c>
-      <c r="L7" s="1">
-        <v>0</v>
-      </c>
-      <c r="M7" s="1"/>
+      <c r="M7" s="1">
+        <v>1</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B8" s="1">
+        <f t="shared" si="0"/>
+        <v>61503</v>
+      </c>
+      <c r="C8" s="1">
         <v>7542</v>
       </c>
-      <c r="C8" s="1">
+      <c r="D8" s="1">
         <v>28475</v>
       </c>
-      <c r="D8" s="1">
+      <c r="E8" s="1">
         <v>25486</v>
       </c>
-      <c r="E8" s="1">
+      <c r="F8" s="1">
         <v>1900</v>
       </c>
-      <c r="F8" s="1">
+      <c r="G8" s="1">
         <v>362</v>
       </c>
-      <c r="G8" s="2">
+      <c r="H8" s="4">
         <v>2015</v>
       </c>
-      <c r="H8" s="1">
+      <c r="I8" s="1">
         <v>2425</v>
       </c>
-      <c r="I8" s="1">
+      <c r="J8" s="1">
         <v>553</v>
       </c>
-      <c r="J8" s="1">
+      <c r="K8" s="1">
         <v>594</v>
       </c>
-      <c r="K8" s="1">
+      <c r="L8" s="1">
         <v>1072</v>
       </c>
-      <c r="L8" s="1">
+      <c r="M8" s="1">
         <v>883</v>
       </c>
-      <c r="M8" s="1">
+      <c r="N8" s="1">
         <v>1508</v>
       </c>
+      <c r="O8" s="1">
+        <v>2</v>
+      </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B9" s="1">
+        <f t="shared" si="0"/>
+        <v>57620</v>
+      </c>
+      <c r="C9" s="1">
         <v>7412</v>
       </c>
-      <c r="C9" s="1">
+      <c r="D9" s="1">
         <v>26375</v>
       </c>
-      <c r="D9" s="1">
+      <c r="E9" s="1">
         <v>23833</v>
       </c>
-      <c r="E9" s="1">
+      <c r="F9" s="1">
         <v>1900</v>
       </c>
-      <c r="F9" s="1">
+      <c r="G9" s="1">
         <v>351</v>
       </c>
-      <c r="G9" s="2">
+      <c r="H9" s="4">
         <v>1985</v>
       </c>
-      <c r="H9" s="1">
+      <c r="I9" s="1">
         <v>2347</v>
       </c>
-      <c r="I9" s="1">
+      <c r="J9" s="1">
         <v>553</v>
       </c>
-      <c r="J9" s="1">
+      <c r="K9" s="1">
         <v>594</v>
       </c>
-      <c r="K9" s="1">
+      <c r="L9" s="1">
         <v>1066</v>
       </c>
-      <c r="L9" s="1">
+      <c r="M9" s="1">
         <v>867</v>
       </c>
-      <c r="M9" s="1">
+      <c r="N9" s="1">
         <v>1483</v>
       </c>
+      <c r="O9" s="1">
+        <v>2</v>
+      </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B10" s="1">
+        <f t="shared" si="0"/>
+        <v>47150</v>
+      </c>
+      <c r="C10" s="1">
         <v>5970</v>
       </c>
-      <c r="C10" s="1">
+      <c r="D10" s="1">
         <v>22028</v>
       </c>
-      <c r="D10" s="1">
+      <c r="E10" s="1">
         <v>19152</v>
       </c>
-      <c r="E10" s="1">
+      <c r="F10" s="1">
         <v>1900</v>
       </c>
-      <c r="F10" s="1">
+      <c r="G10" s="1">
         <v>363</v>
       </c>
-      <c r="G10" s="2">
+      <c r="H10" s="4">
         <v>1877</v>
       </c>
-      <c r="H10" s="1">
+      <c r="I10" s="1">
         <v>1125</v>
       </c>
-      <c r="I10" s="1">
+      <c r="J10" s="1">
         <v>553</v>
       </c>
-      <c r="J10" s="1">
+      <c r="K10" s="1">
         <v>594</v>
       </c>
-      <c r="K10" s="1">
+      <c r="L10" s="1">
         <v>1049</v>
       </c>
-      <c r="L10" s="1">
+      <c r="M10" s="1">
         <v>772</v>
       </c>
-      <c r="M10" s="1">
+      <c r="N10" s="1">
         <v>1194</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="1">
+        <f t="shared" si="0"/>
+        <v>45180</v>
+      </c>
+      <c r="C11" s="1">
         <v>5912</v>
       </c>
-      <c r="C11" s="1">
+      <c r="D11" s="1">
         <v>20956</v>
       </c>
-      <c r="D11" s="1">
+      <c r="E11" s="1">
         <v>18312</v>
       </c>
-      <c r="E11" s="1">
+      <c r="F11" s="1">
         <v>1900</v>
       </c>
-      <c r="F11" s="1">
+      <c r="G11" s="1">
         <v>363</v>
       </c>
-      <c r="G11" s="2">
+      <c r="H11" s="4">
         <v>1860</v>
       </c>
-      <c r="H11" s="1">
+      <c r="I11" s="1">
         <v>1095</v>
       </c>
-      <c r="I11" s="1">
+      <c r="J11" s="1">
         <v>553</v>
       </c>
-      <c r="J11" s="1">
+      <c r="K11" s="1">
         <v>594</v>
       </c>
-      <c r="K11" s="1">
+      <c r="L11" s="1">
         <v>1046</v>
       </c>
-      <c r="L11" s="1">
+      <c r="M11" s="1">
         <v>764</v>
       </c>
-      <c r="M11" s="1">
+      <c r="N11" s="1">
         <v>1182</v>
+      </c>
+      <c r="O11" s="1">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="1">
+        <f t="shared" si="0"/>
+        <v>11180</v>
+      </c>
+      <c r="C12" s="1">
+        <v>6503</v>
+      </c>
+      <c r="D12" s="1">
+        <v>229</v>
+      </c>
+      <c r="E12" s="1">
+        <v>4448</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G12" s="1">
+        <v>450</v>
+      </c>
+      <c r="H12" s="1">
+        <v>1186.3399999999999</v>
+      </c>
+      <c r="I12" s="1">
+        <v>918.21</v>
+      </c>
+      <c r="J12" s="1">
+        <v>663</v>
+      </c>
+      <c r="K12" s="1">
+        <v>258.7</v>
+      </c>
+      <c r="L12" s="1">
+        <v>459.04</v>
+      </c>
+      <c r="M12" s="1">
+        <v>1</v>
+      </c>
+      <c r="N12" s="1">
+        <v>472</v>
+      </c>
+      <c r="O12" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="1">
+        <f t="shared" si="0"/>
+        <v>83417</v>
+      </c>
+      <c r="C13" s="1">
+        <v>10747</v>
+      </c>
+      <c r="D13" s="1">
+        <v>22074</v>
+      </c>
+      <c r="E13" s="1">
+        <v>50596</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G13" s="1">
+        <v>450</v>
+      </c>
+      <c r="H13" s="1">
+        <v>453</v>
+      </c>
+      <c r="I13" s="1">
+        <v>2969</v>
+      </c>
+      <c r="J13" s="1">
+        <v>288</v>
+      </c>
+      <c r="K13" s="1">
+        <v>519</v>
+      </c>
+      <c r="L13" s="1">
+        <v>56</v>
+      </c>
+      <c r="M13" s="1">
+        <v>527</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="O13" s="1">
+        <v>3</v>
+      </c>
+      <c r="P13">
+        <f>O13*8.3</f>
+        <v>24.900000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>